<commit_message>
docs: update dermaesthetic mvp gantt chart
</commit_message>
<xml_diff>
--- a/docs/superpowers/specs/v1/dermaesthetic-mvp-gantt.xlsx
+++ b/docs/superpowers/specs/v1/dermaesthetic-mvp-gantt.xlsx
@@ -27,12 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="195">
   <si>
     <t>Dermaesthetic Super Apps - MVP Gantt Chart</t>
   </si>
   <si>
-    <t>Timeline: June 2026 - March 2027 | Team: 2 Flutter Devs + 2 Fullstack Devs</t>
+    <t>Timeline: June 2026 - February 2027 | Team: 2 Flutter Devs + 2 Fullstack Devs</t>
   </si>
   <si>
     <t>Sprint</t>
@@ -173,23 +173,23 @@
   </si>
   <si>
     <t>W30
-Mar 08</t>
+Jan 11</t>
   </si>
   <si>
     <t>W31
-Mar 15</t>
+Jan 18</t>
   </si>
   <si>
     <t>W32
-Mar 22</t>
+Jan 25</t>
   </si>
   <si>
     <t>W33
-Mar 29</t>
+Feb 1</t>
   </si>
   <si>
     <t>W34
-Apr 05</t>
+Feb 8</t>
   </si>
   <si>
     <t>B-1</t>
@@ -216,7 +216,7 @@
     <t>Core APIs</t>
   </si>
   <si>
-    <t>Brand, Booking, Promotion APIs</t>
+    <t>Brand Clinic, Booking, Promotion APIs</t>
   </si>
   <si>
     <t>2026-06-29</t>
@@ -372,7 +372,7 @@
     <t>Multi Language</t>
   </si>
   <si>
-    <t>Language selection, EN/ID/JP strings, Locale persistence, Dynamic UI labels</t>
+    <t>Language selection, EN/ID strings, Locale persistence, Dynamic UI labels</t>
   </si>
   <si>
     <t>M-3</t>
@@ -483,7 +483,7 @@
     <t>History &amp; Skin</t>
   </si>
   <si>
-    <t>Booking history, Skin analysis questionnaire, Saved patients in timeline</t>
+    <t>Booking history, Skin analysis questionnaire, Saved patients</t>
   </si>
   <si>
     <t>M-14</t>
@@ -634,9 +634,6 @@
   </si>
   <si>
     <t>LEGEND</t>
-  </si>
-  <si>
-    <t>█</t>
   </si>
   <si>
     <t>Backend Development</t>
@@ -662,7 +659,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -690,14 +687,6 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -895,7 +884,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -912,12 +901,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
         <bgColor rgb="FF4472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2F5496"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -1285,52 +1268,55 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="13" borderId="0">
@@ -1345,89 +1331,86 @@
     <xf numFmtId="0" fontId="30" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="33" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="34" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="37" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="38" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="39" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1435,34 +1418,31 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1825,11 +1805,91 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:41">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
+      <c r="AF2" s="2"/>
+      <c r="AG2" s="2"/>
+      <c r="AH2" s="2"/>
+      <c r="AI2" s="2"/>
+      <c r="AJ2" s="2"/>
+      <c r="AK2" s="2"/>
+      <c r="AL2" s="2"/>
+      <c r="AM2" s="2"/>
+      <c r="AN2" s="2"/>
+      <c r="AO2" s="2"/>
     </row>
     <row r="4" ht="40" customHeight="1" spans="1:41">
       <c r="A4" s="3" t="s">
@@ -1940,261 +2000,261 @@
       <c r="AJ4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="AK4" s="4" t="s">
+      <c r="AK4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AL4" s="4" t="s">
+      <c r="AL4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AM4" s="4" t="s">
+      <c r="AM4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AN4" s="4" t="s">
+      <c r="AN4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="AO4" s="4" t="s">
+      <c r="AO4" s="3" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" ht="28" spans="1:41">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>1</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="9"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" ht="28" spans="1:41">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <v>2</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="I6" s="9"/>
+      <c r="I6" s="8"/>
     </row>
     <row r="7" spans="1:41">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <v>3</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="J7" s="9"/>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" ht="28" spans="1:41">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>4</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="K8" s="9"/>
+      <c r="K8" s="8"/>
     </row>
     <row r="9" ht="28" spans="1:41">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="5">
         <v>5</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="L9" s="9"/>
+      <c r="L9" s="8"/>
     </row>
     <row r="10" ht="28" spans="1:41">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="5">
         <v>6</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="M10" s="9"/>
+      <c r="M10" s="8"/>
     </row>
     <row r="11" ht="28" spans="1:41">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="5">
         <v>7</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="N11" s="9"/>
+      <c r="N11" s="8"/>
     </row>
     <row r="12" ht="28" spans="1:41">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="5">
         <v>8</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="O12" s="9"/>
+      <c r="O12" s="8"/>
     </row>
     <row r="13" ht="44" spans="1:41">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="5">
         <v>9</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="P13" s="10"/>
+      <c r="P13" s="9"/>
     </row>
     <row r="14" ht="44" spans="1:41">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="5">
         <v>10</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="Q14" s="10"/>
+      <c r="Q14" s="9"/>
     </row>
     <row r="15" ht="41" spans="1:41">
       <c r="A15" t="s">
@@ -2203,23 +2263,23 @@
       <c r="B15" t="s">
         <v>93</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <v>2</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="10">
         <v>46202</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="10">
         <v>46208</v>
       </c>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
     </row>
     <row r="16" ht="28" spans="1:41">
       <c r="A16" t="s">
@@ -2228,718 +2288,695 @@
       <c r="B16" t="s">
         <v>93</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <v>4</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="10">
         <v>46216</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="10">
         <v>46222</v>
       </c>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
-    </row>
-    <row r="17" ht="41" spans="1:29">
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+    </row>
+    <row r="17" ht="41" spans="1:28">
       <c r="A17" t="s">
         <v>98</v>
       </c>
       <c r="B17" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="5">
         <v>6</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="10">
         <v>46230</v>
       </c>
-      <c r="G17" s="11">
+      <c r="G17" s="10">
         <v>46236</v>
       </c>
-      <c r="M17" s="12"/>
-      <c r="N17" s="12"/>
-    </row>
-    <row r="18" ht="41" spans="1:29">
+      <c r="M17" s="11"/>
+    </row>
+    <row r="18" ht="41" spans="1:28">
       <c r="A18" t="s">
         <v>101</v>
       </c>
       <c r="B18" t="s">
         <v>93</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="5">
         <v>7</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="10">
         <v>46237</v>
       </c>
-      <c r="G18" s="11">
+      <c r="G18" s="10">
         <v>46243</v>
       </c>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-    </row>
-    <row r="19" ht="28" spans="1:29">
-      <c r="A19" s="5" t="s">
+      <c r="N18" s="11"/>
+    </row>
+    <row r="19" ht="28" spans="1:28">
+      <c r="A19" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="5">
         <v>8</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F19" s="13">
+      <c r="F19" s="12">
         <v>46244</v>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="12">
         <v>46250</v>
       </c>
-      <c r="O19" s="12"/>
-      <c r="P19" s="12"/>
-    </row>
-    <row r="20" ht="28" spans="1:29">
-      <c r="A20" s="5" t="s">
+      <c r="O19" s="11"/>
+    </row>
+    <row r="20" ht="28" spans="1:28">
+      <c r="A20" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="5">
         <v>9</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="F20" s="13">
+      <c r="F20" s="12">
         <v>46251</v>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="12">
         <v>46257</v>
       </c>
-      <c r="P20" s="12"/>
-      <c r="Q20" s="12"/>
-    </row>
-    <row r="21" spans="1:29">
-      <c r="A21" s="5" t="s">
+      <c r="P20" s="11"/>
+    </row>
+    <row r="21" spans="1:28">
+      <c r="A21" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="5">
         <v>10</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F21" s="13">
+      <c r="F21" s="12">
         <v>46258</v>
       </c>
-      <c r="G21" s="13">
+      <c r="G21" s="12">
         <v>46264</v>
       </c>
-      <c r="Q21" s="12"/>
-      <c r="R21" s="12"/>
-    </row>
-    <row r="22" spans="1:29">
-      <c r="A22" s="5" t="s">
+      <c r="Q21" s="11"/>
+    </row>
+    <row r="22" spans="1:28">
+      <c r="A22" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="5">
         <v>11</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="12">
         <v>46265</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="12">
         <v>46271</v>
       </c>
-      <c r="R22" s="12"/>
-      <c r="S22" s="12"/>
-    </row>
-    <row r="23" ht="28" spans="1:29">
-      <c r="A23" s="5" t="s">
+      <c r="R22" s="11"/>
+    </row>
+    <row r="23" ht="28" spans="1:28">
+      <c r="A23" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <v>12</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="12">
         <v>46272</v>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="12">
         <v>46278</v>
       </c>
-      <c r="S23" s="12"/>
-      <c r="T23" s="12"/>
-    </row>
-    <row r="24" ht="28" spans="1:29">
-      <c r="A24" s="5" t="s">
+      <c r="S23" s="11"/>
+    </row>
+    <row r="24" ht="28" spans="1:28">
+      <c r="A24" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <v>13</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="12">
         <v>46279</v>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="12">
         <v>46285</v>
       </c>
-      <c r="T24" s="12"/>
-      <c r="U24" s="12"/>
-    </row>
-    <row r="25" ht="28" customHeight="1" spans="1:29">
-      <c r="A25" s="5" t="s">
+      <c r="T24" s="11"/>
+    </row>
+    <row r="25" ht="28" customHeight="1" spans="1:28">
+      <c r="A25" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <v>14</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="F25" s="13">
+      <c r="F25" s="12">
         <v>46286</v>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="12">
         <v>46292</v>
       </c>
-      <c r="U25" s="12"/>
-      <c r="V25" s="12"/>
-    </row>
-    <row r="26" ht="41" spans="1:29">
-      <c r="A26" s="5" t="s">
+      <c r="U25" s="11"/>
+    </row>
+    <row r="26" ht="41" spans="1:28">
+      <c r="A26" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="5">
         <v>15</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F26" s="13">
+      <c r="F26" s="12">
         <v>46293</v>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="12">
         <v>46299</v>
       </c>
-      <c r="V26" s="14"/>
-    </row>
-    <row r="27" ht="29" spans="1:29">
-      <c r="A27" s="5" t="s">
+      <c r="V26" s="13"/>
+    </row>
+    <row r="27" ht="29" spans="1:28">
+      <c r="A27" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="5">
         <v>16</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="F27" s="13">
+      <c r="F27" s="12">
         <v>46300</v>
       </c>
-      <c r="G27" s="13">
+      <c r="G27" s="12">
         <v>46306</v>
       </c>
-      <c r="W27" s="12"/>
-      <c r="X27" s="12"/>
-    </row>
-    <row r="28" ht="29" spans="1:29">
-      <c r="A28" s="5" t="s">
+      <c r="W27" s="11"/>
+    </row>
+    <row r="28" ht="29" spans="1:28">
+      <c r="A28" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="5">
         <v>17</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="F28" s="13">
+      <c r="F28" s="12">
         <v>46307</v>
       </c>
-      <c r="G28" s="13">
+      <c r="G28" s="12">
         <v>46313</v>
       </c>
-      <c r="X28" s="12"/>
-      <c r="Y28" s="12"/>
-    </row>
-    <row r="29" ht="29" spans="1:29">
-      <c r="A29" s="5" t="s">
+      <c r="X28" s="11"/>
+    </row>
+    <row r="29" ht="29" spans="1:28">
+      <c r="A29" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="5">
         <v>18</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="F29" s="13">
+      <c r="F29" s="12">
         <v>46314</v>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="12">
         <v>46320</v>
       </c>
-      <c r="Y29" s="14"/>
-    </row>
-    <row r="30" ht="29" spans="1:29">
-      <c r="A30" s="5" t="s">
+      <c r="Y29" s="13"/>
+    </row>
+    <row r="30" ht="29" spans="1:28">
+      <c r="A30" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="5">
         <v>19</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F30" s="13">
+      <c r="F30" s="12">
         <v>46321</v>
       </c>
-      <c r="G30" s="13">
+      <c r="G30" s="12">
         <v>46327</v>
       </c>
-      <c r="Z30" s="12"/>
-      <c r="AA30" s="12"/>
-    </row>
-    <row r="31" ht="41" spans="1:29">
-      <c r="A31" s="5" t="s">
+      <c r="Z30" s="11"/>
+    </row>
+    <row r="31" ht="29" spans="1:28">
+      <c r="A31" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="5">
         <v>20</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="F31" s="13">
+      <c r="F31" s="12">
         <v>46328</v>
       </c>
-      <c r="G31" s="13">
+      <c r="G31" s="12">
         <v>46334</v>
       </c>
-      <c r="AA31" s="12"/>
-      <c r="AB31" s="12"/>
-    </row>
-    <row r="32" ht="29" spans="1:29">
-      <c r="A32" s="5" t="s">
+      <c r="AA31" s="11"/>
+    </row>
+    <row r="32" ht="29" spans="1:28">
+      <c r="A32" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="5">
         <v>21</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E32" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="F32" s="13">
+      <c r="F32" s="12">
         <v>46335</v>
       </c>
-      <c r="G32" s="13">
+      <c r="G32" s="12">
         <v>46341</v>
       </c>
-      <c r="AB32" s="12"/>
-      <c r="AC32" s="12"/>
+      <c r="AB32" s="11"/>
     </row>
     <row r="33" ht="29" spans="1:41">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="5">
         <v>22</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="F33" s="13">
+      <c r="F33" s="12">
         <v>46342</v>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="12">
         <v>46348</v>
       </c>
-      <c r="AC33" s="12"/>
-      <c r="AD33" s="12"/>
+      <c r="AC33" s="11"/>
     </row>
     <row r="34" ht="29" spans="1:41">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C34" s="5">
         <v>23</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="F34" s="13">
+      <c r="F34" s="12">
         <v>46349</v>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="12">
         <v>46355</v>
       </c>
-      <c r="AD34" s="12"/>
-      <c r="AE34" s="12"/>
+      <c r="AD34" s="11"/>
     </row>
     <row r="35" ht="28" customHeight="1" spans="1:41">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="5">
         <v>24</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="F35" s="13">
+      <c r="F35" s="12">
         <v>46356</v>
       </c>
-      <c r="G35" s="13">
+      <c r="G35" s="12">
         <v>46362</v>
       </c>
-      <c r="AE35" s="12"/>
-      <c r="AF35" s="12"/>
+      <c r="AE35" s="11"/>
     </row>
     <row r="36" ht="41" spans="1:41">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C36" s="6">
+      <c r="C36" s="5">
         <v>25</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="E36" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="F36" s="13">
+      <c r="F36" s="12">
         <v>46363</v>
       </c>
-      <c r="G36" s="13">
+      <c r="G36" s="12">
         <v>46369</v>
       </c>
-      <c r="AF36" s="14"/>
+      <c r="AF36" s="13"/>
     </row>
     <row r="37" ht="29" spans="1:41">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="5">
         <v>26</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E37" s="7" t="s">
+      <c r="E37" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="F37" s="13">
+      <c r="F37" s="12">
         <v>46370</v>
       </c>
-      <c r="G37" s="13">
+      <c r="G37" s="12">
         <v>46376</v>
       </c>
-      <c r="AG37" s="12"/>
-      <c r="AH37" s="12"/>
+      <c r="AG37" s="11"/>
     </row>
     <row r="38" ht="29" spans="1:41">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C38" s="6">
+      <c r="C38" s="5">
         <v>27</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="F38" s="13">
+      <c r="F38" s="12">
         <v>46377</v>
       </c>
-      <c r="G38" s="13">
+      <c r="G38" s="12">
         <v>46383</v>
       </c>
-      <c r="AH38" s="12"/>
-      <c r="AI38" s="12"/>
+      <c r="AH38" s="11"/>
     </row>
     <row r="39" ht="29" spans="1:41">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C39" s="6">
+      <c r="C39" s="5">
         <v>28</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="F39" s="13">
+      <c r="F39" s="12">
         <v>46384</v>
       </c>
-      <c r="G39" s="13">
+      <c r="G39" s="12">
         <v>46390</v>
       </c>
-      <c r="AI39" s="14"/>
+      <c r="AI39" s="13"/>
     </row>
     <row r="40" ht="29" spans="1:41">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C40" s="5">
         <v>29</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="F40" s="13">
+      <c r="F40" s="12">
         <v>46391</v>
       </c>
-      <c r="G40" s="13">
+      <c r="G40" s="12">
         <v>46397</v>
       </c>
-      <c r="AJ40" s="12"/>
-      <c r="AK40" s="12"/>
+      <c r="AJ40" s="11"/>
     </row>
     <row r="41" ht="29" spans="1:41">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C41" s="6">
+      <c r="C41" s="5">
         <v>30</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D41" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="F41" s="13">
+      <c r="F41" s="12">
         <v>46398</v>
       </c>
-      <c r="G41" s="13">
+      <c r="G41" s="12">
         <v>46404</v>
       </c>
-      <c r="AK41" s="12"/>
-      <c r="AL41" s="12"/>
+      <c r="AK41" s="11"/>
     </row>
     <row r="42" ht="29" spans="1:41">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C42" s="6">
+      <c r="C42" s="5">
         <v>31</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="F42" s="13">
+      <c r="F42" s="12">
         <v>46405</v>
       </c>
-      <c r="G42" s="13">
+      <c r="G42" s="12">
         <v>46411</v>
       </c>
-      <c r="AL42" s="12"/>
-      <c r="AM42" s="12"/>
+      <c r="AL42" s="11"/>
     </row>
     <row r="43" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C43" s="6">
+      <c r="C43" s="5">
         <v>32</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D43" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E43" s="7" t="s">
+      <c r="E43" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="F43" s="13">
+      <c r="F43" s="12">
         <v>46412</v>
       </c>
-      <c r="G43" s="13">
+      <c r="G43" s="12">
         <v>46418</v>
       </c>
-      <c r="AM43" s="12"/>
-      <c r="AN43" s="12"/>
+      <c r="AM43" s="11"/>
     </row>
     <row r="44" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C44" s="6">
+      <c r="C44" s="5">
         <v>33</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D44" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="F44" s="13">
+      <c r="F44" s="12">
         <v>46419</v>
       </c>
-      <c r="G44" s="13">
+      <c r="G44" s="12">
         <v>46425</v>
       </c>
-      <c r="AN44" s="14"/>
+      <c r="AN44" s="13"/>
     </row>
     <row r="45" ht="17.6" customHeight="1" spans="1:41">
       <c r="A45" t="s">
@@ -2948,696 +2985,690 @@
       <c r="B45" t="s">
         <v>93</v>
       </c>
-      <c r="C45" s="15">
+      <c r="C45" s="14">
         <v>34</v>
       </c>
-      <c r="D45" s="16" t="s">
+      <c r="D45" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="E45" s="17" t="s">
+      <c r="E45" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="F45" s="11">
+      <c r="F45" s="10">
         <v>46426</v>
       </c>
-      <c r="G45" s="11">
+      <c r="G45" s="10">
         <v>46432</v>
       </c>
-      <c r="AO45" s="14"/>
+      <c r="AO45" s="13"/>
     </row>
     <row r="46" ht="17.6" customHeight="1"/>
     <row r="47" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A47" s="18" t="s">
+      <c r="A47" s="17" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="48" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20" t="s">
+      <c r="B48" s="19"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19" t="s">
         <v>182</v>
       </c>
-      <c r="F48" s="21">
+      <c r="F48" s="20">
         <v>46223</v>
       </c>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="20"/>
-      <c r="J48" s="20"/>
-      <c r="K48" s="20"/>
-      <c r="L48" s="19" t="s">
+      <c r="G48" s="19"/>
+      <c r="H48" s="19"/>
+      <c r="I48" s="19"/>
+      <c r="J48" s="19"/>
+      <c r="K48" s="19"/>
+      <c r="L48" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="M48" s="20"/>
-      <c r="N48" s="20"/>
-      <c r="O48" s="20"/>
-      <c r="P48" s="20"/>
-      <c r="Q48" s="20"/>
-      <c r="R48" s="20"/>
-      <c r="S48" s="20"/>
-      <c r="T48" s="20"/>
-      <c r="U48" s="20"/>
-      <c r="V48" s="20"/>
-      <c r="W48" s="20"/>
-      <c r="X48" s="20"/>
-      <c r="Y48" s="20"/>
-      <c r="Z48" s="20"/>
-      <c r="AA48" s="20"/>
-      <c r="AB48" s="20"/>
-      <c r="AC48" s="20"/>
-      <c r="AD48" s="20"/>
+      <c r="M48" s="19"/>
+      <c r="N48" s="19"/>
+      <c r="O48" s="19"/>
+      <c r="P48" s="19"/>
+      <c r="Q48" s="19"/>
+      <c r="R48" s="19"/>
+      <c r="S48" s="19"/>
+      <c r="T48" s="19"/>
+      <c r="U48" s="19"/>
+      <c r="V48" s="19"/>
+      <c r="W48" s="19"/>
+      <c r="X48" s="19"/>
+      <c r="Y48" s="19"/>
+      <c r="Z48" s="19"/>
+      <c r="AA48" s="19"/>
+      <c r="AB48" s="19"/>
+      <c r="AC48" s="19"/>
+      <c r="AD48" s="19"/>
       <c r="AE48"/>
       <c r="AF48"/>
       <c r="AG48"/>
       <c r="AH48"/>
-      <c r="AI48" s="20"/>
-      <c r="AJ48" s="20"/>
-      <c r="AK48" s="20"/>
+      <c r="AI48" s="19"/>
+      <c r="AJ48" s="19"/>
+      <c r="AK48" s="19"/>
     </row>
     <row r="49" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A49" s="19" t="s">
+      <c r="A49" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20" t="s">
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="F49" s="21">
+      <c r="F49" s="20">
         <v>46244</v>
       </c>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20"/>
-      <c r="I49" s="20"/>
-      <c r="J49" s="20"/>
-      <c r="K49" s="20"/>
-      <c r="L49" s="20"/>
-      <c r="M49" s="20"/>
-      <c r="N49" s="20"/>
-      <c r="O49" s="20"/>
-      <c r="P49" s="19" t="s">
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
+      <c r="J49" s="19"/>
+      <c r="K49" s="19"/>
+      <c r="L49" s="19"/>
+      <c r="M49" s="19"/>
+      <c r="N49" s="19"/>
+      <c r="O49" s="19"/>
+      <c r="P49" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="Q49" s="20"/>
-      <c r="R49" s="20"/>
-      <c r="S49" s="20"/>
-      <c r="T49" s="20"/>
-      <c r="U49" s="20"/>
-      <c r="V49" s="20"/>
-      <c r="W49" s="20"/>
-      <c r="X49" s="20"/>
-      <c r="Y49" s="20"/>
-      <c r="Z49" s="20"/>
-      <c r="AA49" s="20"/>
-      <c r="AB49" s="20"/>
-      <c r="AC49" s="20"/>
-      <c r="AD49" s="20"/>
+      <c r="Q49" s="19"/>
+      <c r="R49" s="19"/>
+      <c r="S49" s="19"/>
+      <c r="T49" s="19"/>
+      <c r="U49" s="19"/>
+      <c r="V49" s="19"/>
+      <c r="W49" s="19"/>
+      <c r="X49" s="19"/>
+      <c r="Y49" s="19"/>
+      <c r="Z49" s="19"/>
+      <c r="AA49" s="19"/>
+      <c r="AB49" s="19"/>
+      <c r="AC49" s="19"/>
+      <c r="AD49" s="19"/>
       <c r="AE49"/>
       <c r="AF49"/>
       <c r="AG49"/>
       <c r="AH49"/>
-      <c r="AI49" s="20"/>
-      <c r="AJ49" s="20"/>
-      <c r="AK49" s="20"/>
+      <c r="AI49" s="19"/>
+      <c r="AJ49" s="19"/>
+      <c r="AK49" s="19"/>
     </row>
     <row r="50" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A50" s="19" t="s">
+      <c r="A50" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="20" t="s">
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="F50" s="21">
+      <c r="F50" s="20">
         <v>46258</v>
       </c>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20"/>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20"/>
-      <c r="L50" s="20"/>
-      <c r="M50" s="20"/>
-      <c r="N50" s="20"/>
-      <c r="O50" s="20"/>
-      <c r="P50" s="20"/>
-      <c r="Q50" s="19" t="s">
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
+      <c r="K50" s="19"/>
+      <c r="L50" s="19"/>
+      <c r="M50" s="19"/>
+      <c r="N50" s="19"/>
+      <c r="O50" s="19"/>
+      <c r="P50" s="19"/>
+      <c r="Q50" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="R50" s="20"/>
-      <c r="S50" s="20"/>
-      <c r="T50" s="20"/>
-      <c r="U50" s="20"/>
-      <c r="V50" s="20"/>
-      <c r="W50" s="20"/>
-      <c r="X50" s="20"/>
-      <c r="Y50" s="20"/>
-      <c r="Z50" s="20"/>
-      <c r="AA50" s="20"/>
-      <c r="AB50" s="20"/>
-      <c r="AC50" s="20"/>
-      <c r="AD50" s="20"/>
+      <c r="R50" s="19"/>
+      <c r="S50" s="19"/>
+      <c r="T50" s="19"/>
+      <c r="U50" s="19"/>
+      <c r="V50" s="19"/>
+      <c r="W50" s="19"/>
+      <c r="X50" s="19"/>
+      <c r="Y50" s="19"/>
+      <c r="Z50" s="19"/>
+      <c r="AA50" s="19"/>
+      <c r="AB50" s="19"/>
+      <c r="AC50" s="19"/>
+      <c r="AD50" s="19"/>
       <c r="AE50"/>
       <c r="AF50"/>
       <c r="AG50"/>
       <c r="AH50"/>
-      <c r="AI50" s="20"/>
-      <c r="AJ50" s="20"/>
-      <c r="AK50" s="20"/>
+      <c r="AI50" s="19"/>
+      <c r="AJ50" s="19"/>
+      <c r="AK50" s="19"/>
     </row>
     <row r="51" spans="1:41">
-      <c r="A51" s="19" t="s">
+      <c r="A51" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B51" s="20"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="20" t="s">
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="F51" s="21">
+      <c r="F51" s="20">
         <v>46300</v>
       </c>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
-      <c r="L51" s="20"/>
-      <c r="M51" s="20"/>
-      <c r="N51" s="20"/>
-      <c r="O51" s="20"/>
-      <c r="P51" s="20"/>
-      <c r="Q51" s="20"/>
-      <c r="R51" s="20"/>
-      <c r="S51" s="20"/>
-      <c r="T51" s="20"/>
-      <c r="U51" s="20"/>
-      <c r="V51" s="20"/>
-      <c r="W51" s="19" t="s">
+      <c r="G51" s="19"/>
+      <c r="H51" s="19"/>
+      <c r="I51" s="19"/>
+      <c r="J51" s="19"/>
+      <c r="K51" s="19"/>
+      <c r="L51" s="19"/>
+      <c r="M51" s="19"/>
+      <c r="N51" s="19"/>
+      <c r="O51" s="19"/>
+      <c r="P51" s="19"/>
+      <c r="Q51" s="19"/>
+      <c r="R51" s="19"/>
+      <c r="S51" s="19"/>
+      <c r="T51" s="19"/>
+      <c r="U51" s="19"/>
+      <c r="V51" s="19"/>
+      <c r="W51" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="X51" s="20"/>
-      <c r="Y51" s="20"/>
-      <c r="Z51" s="20"/>
-      <c r="AA51" s="20"/>
-      <c r="AB51" s="20"/>
-      <c r="AC51" s="20"/>
-      <c r="AD51" s="20"/>
-      <c r="AE51" s="20"/>
-      <c r="AF51" s="20"/>
-      <c r="AG51" s="20"/>
-      <c r="AH51" s="20"/>
-      <c r="AI51" s="20"/>
-      <c r="AJ51" s="20"/>
-      <c r="AK51" s="20"/>
+      <c r="X51" s="19"/>
+      <c r="Y51" s="19"/>
+      <c r="Z51" s="19"/>
+      <c r="AA51" s="19"/>
+      <c r="AB51" s="19"/>
+      <c r="AC51" s="19"/>
+      <c r="AD51" s="19"/>
+      <c r="AE51" s="19"/>
+      <c r="AF51" s="19"/>
+      <c r="AG51" s="19"/>
+      <c r="AH51" s="19"/>
+      <c r="AI51" s="19"/>
+      <c r="AJ51" s="19"/>
+      <c r="AK51" s="19"/>
     </row>
     <row r="52" spans="1:41">
-      <c r="A52" s="19" t="s">
+      <c r="A52" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B52" s="20"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20" t="s">
+      <c r="B52" s="19"/>
+      <c r="C52" s="19"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="F52" s="21">
+      <c r="F52" s="20">
         <v>46321</v>
       </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
-      <c r="L52" s="20"/>
-      <c r="M52" s="20"/>
-      <c r="N52" s="20"/>
-      <c r="O52" s="20"/>
-      <c r="P52" s="20"/>
-      <c r="Q52" s="20"/>
-      <c r="R52" s="20"/>
-      <c r="S52" s="20"/>
-      <c r="T52" s="20"/>
-      <c r="U52" s="20"/>
-      <c r="V52" s="20"/>
-      <c r="W52" s="20"/>
-      <c r="X52" s="20"/>
-      <c r="Y52" s="20"/>
-      <c r="Z52" s="19" t="s">
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+      <c r="Q52" s="19"/>
+      <c r="R52" s="19"/>
+      <c r="S52" s="19"/>
+      <c r="T52" s="19"/>
+      <c r="U52" s="19"/>
+      <c r="V52" s="19"/>
+      <c r="W52" s="19"/>
+      <c r="X52" s="19"/>
+      <c r="Y52" s="19"/>
+      <c r="Z52" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="AA52" s="20"/>
-      <c r="AB52" s="20"/>
-      <c r="AC52" s="20"/>
-      <c r="AD52" s="20"/>
-      <c r="AE52" s="20"/>
-      <c r="AF52" s="20"/>
-      <c r="AG52" s="20"/>
-      <c r="AH52" s="20"/>
-      <c r="AI52" s="20"/>
-      <c r="AJ52" s="20"/>
-      <c r="AK52" s="20"/>
+      <c r="AA52" s="19"/>
+      <c r="AB52" s="19"/>
+      <c r="AC52" s="19"/>
+      <c r="AD52" s="19"/>
+      <c r="AE52" s="19"/>
+      <c r="AF52" s="19"/>
+      <c r="AG52" s="19"/>
+      <c r="AH52" s="19"/>
+      <c r="AI52" s="19"/>
+      <c r="AJ52" s="19"/>
+      <c r="AK52" s="19"/>
     </row>
     <row r="53" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A53" s="19" t="s">
+      <c r="A53" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20" t="s">
+      <c r="B53" s="19"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
+      <c r="E53" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="F53" s="21">
+      <c r="F53" s="20">
         <v>46363</v>
       </c>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20"/>
-      <c r="J53" s="20"/>
-      <c r="K53" s="20"/>
-      <c r="L53" s="20"/>
-      <c r="M53" s="20"/>
-      <c r="N53" s="20"/>
-      <c r="O53" s="20"/>
-      <c r="P53" s="20"/>
-      <c r="Q53" s="20"/>
-      <c r="R53" s="20"/>
-      <c r="S53" s="20"/>
-      <c r="T53" s="20"/>
-      <c r="U53" s="20"/>
-      <c r="V53" s="20"/>
-      <c r="W53" s="20"/>
-      <c r="X53" s="20"/>
-      <c r="Y53" s="20"/>
-      <c r="Z53" s="20"/>
-      <c r="AA53" s="20"/>
-      <c r="AB53" s="20"/>
-      <c r="AC53" s="20"/>
-      <c r="AD53" s="20"/>
-      <c r="AE53" s="20"/>
-      <c r="AF53" s="19" t="s">
+      <c r="G53" s="19"/>
+      <c r="H53" s="19"/>
+      <c r="I53" s="19"/>
+      <c r="J53" s="19"/>
+      <c r="K53" s="19"/>
+      <c r="L53" s="19"/>
+      <c r="M53" s="19"/>
+      <c r="N53" s="19"/>
+      <c r="O53" s="19"/>
+      <c r="P53" s="19"/>
+      <c r="Q53" s="19"/>
+      <c r="R53" s="19"/>
+      <c r="S53" s="19"/>
+      <c r="T53" s="19"/>
+      <c r="U53" s="19"/>
+      <c r="V53" s="19"/>
+      <c r="W53" s="19"/>
+      <c r="X53" s="19"/>
+      <c r="Y53" s="19"/>
+      <c r="Z53" s="19"/>
+      <c r="AA53" s="19"/>
+      <c r="AB53" s="19"/>
+      <c r="AC53" s="19"/>
+      <c r="AD53" s="19"/>
+      <c r="AE53" s="19"/>
+      <c r="AF53" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="AG53" s="20"/>
-      <c r="AH53" s="20"/>
-      <c r="AI53" s="20"/>
-      <c r="AJ53" s="20"/>
-      <c r="AK53" s="20"/>
+      <c r="AG53" s="19"/>
+      <c r="AH53" s="19"/>
+      <c r="AI53" s="19"/>
+      <c r="AJ53" s="19"/>
+      <c r="AK53" s="19"/>
     </row>
     <row r="54" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A54" s="19" t="s">
+      <c r="A54" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20" t="s">
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="F54" s="21">
+      <c r="F54" s="20">
         <v>46412</v>
       </c>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20"/>
-      <c r="J54" s="20"/>
-      <c r="K54" s="20"/>
-      <c r="L54" s="20"/>
-      <c r="M54" s="20"/>
-      <c r="N54" s="20"/>
-      <c r="O54" s="20"/>
-      <c r="P54" s="20"/>
-      <c r="Q54" s="20"/>
-      <c r="R54" s="20"/>
-      <c r="S54" s="20"/>
-      <c r="T54" s="20"/>
-      <c r="U54" s="20"/>
-      <c r="V54" s="20"/>
-      <c r="W54" s="20"/>
-      <c r="X54" s="20"/>
-      <c r="Y54" s="20"/>
-      <c r="Z54" s="20"/>
-      <c r="AA54" s="20"/>
-      <c r="AB54" s="20"/>
-      <c r="AC54" s="20"/>
-      <c r="AD54" s="20"/>
-      <c r="AE54" s="20"/>
-      <c r="AF54" s="20"/>
-      <c r="AG54" s="20"/>
-      <c r="AH54" s="20"/>
-      <c r="AI54" s="20"/>
-      <c r="AJ54" s="20"/>
-      <c r="AK54" s="20"/>
-      <c r="AM54" s="19" t="s">
+      <c r="G54" s="19"/>
+      <c r="H54" s="19"/>
+      <c r="I54" s="19"/>
+      <c r="J54" s="19"/>
+      <c r="K54" s="19"/>
+      <c r="L54" s="19"/>
+      <c r="M54" s="19"/>
+      <c r="N54" s="19"/>
+      <c r="O54" s="19"/>
+      <c r="P54" s="19"/>
+      <c r="Q54" s="19"/>
+      <c r="R54" s="19"/>
+      <c r="S54" s="19"/>
+      <c r="T54" s="19"/>
+      <c r="U54" s="19"/>
+      <c r="V54" s="19"/>
+      <c r="W54" s="19"/>
+      <c r="X54" s="19"/>
+      <c r="Y54" s="19"/>
+      <c r="Z54" s="19"/>
+      <c r="AA54" s="19"/>
+      <c r="AB54" s="19"/>
+      <c r="AC54" s="19"/>
+      <c r="AD54" s="19"/>
+      <c r="AE54" s="19"/>
+      <c r="AF54" s="19"/>
+      <c r="AG54" s="19"/>
+      <c r="AH54" s="19"/>
+      <c r="AI54" s="19"/>
+      <c r="AJ54" s="19"/>
+      <c r="AK54" s="19"/>
+      <c r="AM54" s="18" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="55" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A55" s="19" t="s">
+      <c r="A55" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20" t="s">
+      <c r="B55" s="19"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="19"/>
+      <c r="E55" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F55" s="21">
+      <c r="F55" s="20">
         <v>46426</v>
       </c>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="20"/>
-      <c r="K55" s="20"/>
-      <c r="L55" s="20"/>
-      <c r="M55" s="20"/>
-      <c r="N55" s="20"/>
-      <c r="O55" s="20"/>
-      <c r="P55" s="20"/>
-      <c r="Q55" s="20"/>
-      <c r="R55" s="20"/>
-      <c r="S55" s="20"/>
-      <c r="T55" s="20"/>
-      <c r="U55" s="20"/>
-      <c r="V55" s="20"/>
-      <c r="W55" s="20"/>
-      <c r="X55" s="20"/>
-      <c r="Y55" s="20"/>
-      <c r="Z55" s="20"/>
-      <c r="AA55" s="20"/>
-      <c r="AB55" s="20"/>
-      <c r="AC55" s="20"/>
-      <c r="AD55" s="20"/>
-      <c r="AE55" s="20"/>
-      <c r="AF55" s="20"/>
-      <c r="AG55" s="20"/>
-      <c r="AH55" s="20"/>
-      <c r="AI55" s="20"/>
-      <c r="AJ55" s="20"/>
-      <c r="AK55" s="20"/>
-      <c r="AO55" s="19" t="s">
+      <c r="G55" s="19"/>
+      <c r="H55" s="19"/>
+      <c r="I55" s="19"/>
+      <c r="J55" s="19"/>
+      <c r="K55" s="19"/>
+      <c r="L55" s="19"/>
+      <c r="M55" s="19"/>
+      <c r="N55" s="19"/>
+      <c r="O55" s="19"/>
+      <c r="P55" s="19"/>
+      <c r="Q55" s="19"/>
+      <c r="R55" s="19"/>
+      <c r="S55" s="19"/>
+      <c r="T55" s="19"/>
+      <c r="U55" s="19"/>
+      <c r="V55" s="19"/>
+      <c r="W55" s="19"/>
+      <c r="X55" s="19"/>
+      <c r="Y55" s="19"/>
+      <c r="Z55" s="19"/>
+      <c r="AA55" s="19"/>
+      <c r="AB55" s="19"/>
+      <c r="AC55" s="19"/>
+      <c r="AD55" s="19"/>
+      <c r="AE55" s="19"/>
+      <c r="AF55" s="19"/>
+      <c r="AG55" s="19"/>
+      <c r="AH55" s="19"/>
+      <c r="AI55" s="19"/>
+      <c r="AJ55" s="19"/>
+      <c r="AK55" s="19"/>
+      <c r="AO55" s="18" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="56" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A56" s="20"/>
-      <c r="B56" s="20"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="20"/>
-      <c r="K56" s="20"/>
-      <c r="L56" s="20"/>
-      <c r="M56" s="20"/>
-      <c r="N56" s="20"/>
-      <c r="O56" s="20"/>
-      <c r="P56" s="20"/>
-      <c r="Q56" s="20"/>
-      <c r="R56" s="20"/>
-      <c r="S56" s="20"/>
-      <c r="T56" s="20"/>
-      <c r="U56" s="20"/>
-      <c r="V56" s="20"/>
-      <c r="W56" s="20"/>
-      <c r="X56" s="20"/>
-      <c r="Y56" s="20"/>
-      <c r="Z56" s="20"/>
-      <c r="AA56" s="20"/>
-      <c r="AB56" s="20"/>
-      <c r="AC56" s="20"/>
-      <c r="AD56" s="20"/>
-      <c r="AE56" s="20"/>
-      <c r="AF56" s="20"/>
-      <c r="AG56" s="20"/>
-      <c r="AH56" s="20"/>
-      <c r="AI56" s="20"/>
-      <c r="AJ56" s="20"/>
-      <c r="AK56" s="20"/>
+      <c r="A56" s="19"/>
+      <c r="B56" s="19"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
+      <c r="E56" s="19"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="19"/>
+      <c r="I56" s="19"/>
+      <c r="J56" s="19"/>
+      <c r="K56" s="19"/>
+      <c r="L56" s="19"/>
+      <c r="M56" s="19"/>
+      <c r="N56" s="19"/>
+      <c r="O56" s="19"/>
+      <c r="P56" s="19"/>
+      <c r="Q56" s="19"/>
+      <c r="R56" s="19"/>
+      <c r="S56" s="19"/>
+      <c r="T56" s="19"/>
+      <c r="U56" s="19"/>
+      <c r="V56" s="19"/>
+      <c r="W56" s="19"/>
+      <c r="X56" s="19"/>
+      <c r="Y56" s="19"/>
+      <c r="Z56" s="19"/>
+      <c r="AA56" s="19"/>
+      <c r="AB56" s="19"/>
+      <c r="AC56" s="19"/>
+      <c r="AD56" s="19"/>
+      <c r="AE56" s="19"/>
+      <c r="AF56" s="19"/>
+      <c r="AG56" s="19"/>
+      <c r="AH56" s="19"/>
+      <c r="AI56" s="19"/>
+      <c r="AJ56" s="19"/>
+      <c r="AK56" s="19"/>
     </row>
     <row r="57" ht="17.6" customHeight="1" spans="1:41">
-      <c r="A57" s="18" t="s">
+      <c r="A57" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="20"/>
-      <c r="K57" s="20"/>
-      <c r="L57" s="20"/>
-      <c r="M57" s="20"/>
-      <c r="N57" s="20"/>
-      <c r="O57" s="20"/>
-      <c r="P57" s="20"/>
-      <c r="Q57" s="20"/>
-      <c r="R57" s="20"/>
-      <c r="S57" s="20"/>
-      <c r="T57" s="20"/>
-      <c r="U57" s="20"/>
-      <c r="V57" s="20"/>
-      <c r="W57" s="20"/>
-      <c r="X57" s="20"/>
-      <c r="Y57" s="20"/>
-      <c r="Z57" s="20"/>
-      <c r="AA57" s="20"/>
-      <c r="AB57" s="20"/>
-      <c r="AC57" s="20"/>
-      <c r="AD57" s="20"/>
-      <c r="AE57" s="20"/>
-      <c r="AF57" s="20"/>
-      <c r="AG57" s="20"/>
-      <c r="AH57" s="20"/>
-      <c r="AI57" s="20"/>
-      <c r="AJ57" s="20"/>
-      <c r="AK57" s="20"/>
+      <c r="H57" s="19"/>
+      <c r="I57" s="19"/>
+      <c r="J57" s="19"/>
+      <c r="K57" s="19"/>
+      <c r="L57" s="19"/>
+      <c r="M57" s="19"/>
+      <c r="N57" s="19"/>
+      <c r="O57" s="19"/>
+      <c r="P57" s="19"/>
+      <c r="Q57" s="19"/>
+      <c r="R57" s="19"/>
+      <c r="S57" s="19"/>
+      <c r="T57" s="19"/>
+      <c r="U57" s="19"/>
+      <c r="V57" s="19"/>
+      <c r="W57" s="19"/>
+      <c r="X57" s="19"/>
+      <c r="Y57" s="19"/>
+      <c r="Z57" s="19"/>
+      <c r="AA57" s="19"/>
+      <c r="AB57" s="19"/>
+      <c r="AC57" s="19"/>
+      <c r="AD57" s="19"/>
+      <c r="AE57" s="19"/>
+      <c r="AF57" s="19"/>
+      <c r="AG57" s="19"/>
+      <c r="AH57" s="19"/>
+      <c r="AI57" s="19"/>
+      <c r="AJ57" s="19"/>
+      <c r="AK57" s="19"/>
     </row>
     <row r="58" spans="1:41">
-      <c r="A58" s="22" t="s">
+      <c r="A58" s="21"/>
+      <c r="B58" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B58" s="20" t="s">
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="19"/>
+      <c r="I58" s="19"/>
+      <c r="J58" s="19"/>
+      <c r="K58" s="19"/>
+      <c r="L58" s="19"/>
+      <c r="M58" s="19"/>
+      <c r="N58" s="19"/>
+      <c r="O58" s="19"/>
+      <c r="P58" s="19"/>
+      <c r="Q58" s="19"/>
+      <c r="R58" s="19"/>
+      <c r="S58" s="19"/>
+      <c r="T58" s="19"/>
+      <c r="U58" s="19"/>
+      <c r="V58" s="19"/>
+      <c r="W58" s="19"/>
+      <c r="X58" s="19"/>
+      <c r="Y58" s="19"/>
+      <c r="Z58" s="19"/>
+      <c r="AA58" s="19"/>
+      <c r="AB58" s="19"/>
+      <c r="AC58" s="19"/>
+      <c r="AD58" s="19"/>
+      <c r="AE58" s="19"/>
+      <c r="AF58" s="19"/>
+      <c r="AG58" s="19"/>
+      <c r="AH58" s="19"/>
+      <c r="AI58" s="19"/>
+      <c r="AJ58" s="19"/>
+      <c r="AK58" s="19"/>
+    </row>
+    <row r="59" spans="1:41">
+      <c r="A59" s="22"/>
+      <c r="B59" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="20"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
-      <c r="J58" s="20"/>
-      <c r="K58" s="20"/>
-      <c r="L58" s="20"/>
-      <c r="M58" s="20"/>
-      <c r="N58" s="20"/>
-      <c r="O58" s="20"/>
-      <c r="P58" s="20"/>
-      <c r="Q58" s="20"/>
-      <c r="R58" s="20"/>
-      <c r="S58" s="20"/>
-      <c r="T58" s="20"/>
-      <c r="U58" s="20"/>
-      <c r="V58" s="20"/>
-      <c r="W58" s="20"/>
-      <c r="X58" s="20"/>
-      <c r="Y58" s="20"/>
-      <c r="Z58" s="20"/>
-      <c r="AA58" s="20"/>
-      <c r="AB58" s="20"/>
-      <c r="AC58" s="20"/>
-      <c r="AD58" s="20"/>
-      <c r="AE58" s="20"/>
-      <c r="AF58" s="20"/>
-      <c r="AG58" s="20"/>
-      <c r="AH58" s="20"/>
-      <c r="AI58" s="20"/>
-      <c r="AJ58" s="20"/>
-      <c r="AK58" s="20"/>
-    </row>
-    <row r="59" spans="1:41">
-      <c r="A59" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="B59" s="20" t="s">
+      <c r="C59" s="19"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+      <c r="I59" s="19"/>
+      <c r="J59" s="19"/>
+      <c r="K59" s="19"/>
+      <c r="L59" s="19"/>
+      <c r="M59" s="19"/>
+      <c r="N59" s="19"/>
+      <c r="O59" s="19"/>
+      <c r="P59" s="19"/>
+      <c r="Q59" s="19"/>
+      <c r="R59" s="19"/>
+      <c r="S59" s="19"/>
+      <c r="T59" s="19"/>
+      <c r="U59" s="19"/>
+      <c r="V59" s="19"/>
+      <c r="W59" s="19"/>
+      <c r="X59" s="19"/>
+      <c r="Y59" s="19"/>
+      <c r="Z59" s="19"/>
+      <c r="AA59" s="19"/>
+      <c r="AB59" s="19"/>
+      <c r="AC59" s="19"/>
+      <c r="AD59" s="19"/>
+      <c r="AE59" s="19"/>
+      <c r="AF59" s="19"/>
+      <c r="AG59" s="19"/>
+      <c r="AH59" s="19"/>
+      <c r="AI59" s="19"/>
+      <c r="AJ59" s="19"/>
+      <c r="AK59" s="19"/>
+    </row>
+    <row r="60" spans="1:41">
+      <c r="A60" s="23"/>
+      <c r="B60" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
-      <c r="E59" s="20"/>
-      <c r="F59" s="20"/>
-      <c r="G59" s="20"/>
-      <c r="H59" s="20"/>
-      <c r="I59" s="20"/>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20"/>
-      <c r="L59" s="20"/>
-      <c r="M59" s="20"/>
-      <c r="N59" s="20"/>
-      <c r="O59" s="20"/>
-      <c r="P59" s="20"/>
-      <c r="Q59" s="20"/>
-      <c r="R59" s="20"/>
-      <c r="S59" s="20"/>
-      <c r="T59" s="20"/>
-      <c r="U59" s="20"/>
-      <c r="V59" s="20"/>
-      <c r="W59" s="20"/>
-      <c r="X59" s="20"/>
-      <c r="Y59" s="20"/>
-      <c r="Z59" s="20"/>
-      <c r="AA59" s="20"/>
-      <c r="AB59" s="20"/>
-      <c r="AC59" s="20"/>
-      <c r="AD59" s="20"/>
-      <c r="AE59" s="20"/>
-      <c r="AF59" s="20"/>
-      <c r="AG59" s="20"/>
-      <c r="AH59" s="20"/>
-      <c r="AI59" s="20"/>
-      <c r="AJ59" s="20"/>
-      <c r="AK59" s="20"/>
-    </row>
-    <row r="60" spans="1:41">
-      <c r="A60" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="B60" s="20" t="s">
+      <c r="C60" s="19"/>
+      <c r="D60" s="19"/>
+      <c r="E60" s="19"/>
+      <c r="F60" s="19"/>
+      <c r="G60" s="19"/>
+      <c r="H60" s="19"/>
+      <c r="I60" s="19"/>
+      <c r="J60" s="19"/>
+      <c r="K60" s="19"/>
+      <c r="L60" s="19"/>
+      <c r="M60" s="19"/>
+      <c r="N60" s="19"/>
+      <c r="O60" s="19"/>
+      <c r="P60" s="19"/>
+      <c r="Q60" s="19"/>
+      <c r="R60" s="19"/>
+      <c r="S60" s="19"/>
+      <c r="T60" s="19"/>
+      <c r="U60" s="19"/>
+      <c r="V60" s="19"/>
+      <c r="W60" s="19"/>
+      <c r="X60" s="19"/>
+      <c r="Y60" s="19"/>
+      <c r="Z60" s="19"/>
+      <c r="AA60" s="19"/>
+      <c r="AB60" s="19"/>
+      <c r="AC60" s="19"/>
+      <c r="AD60" s="19"/>
+      <c r="AE60" s="19"/>
+      <c r="AF60" s="19"/>
+      <c r="AG60" s="19"/>
+      <c r="AH60" s="19"/>
+      <c r="AI60" s="19"/>
+      <c r="AJ60" s="19"/>
+      <c r="AK60" s="19"/>
+    </row>
+    <row r="61" spans="1:41">
+      <c r="A61" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="B61" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-      <c r="L60" s="20"/>
-      <c r="M60" s="20"/>
-      <c r="N60" s="20"/>
-      <c r="O60" s="20"/>
-      <c r="P60" s="20"/>
-      <c r="Q60" s="20"/>
-      <c r="R60" s="20"/>
-      <c r="S60" s="20"/>
-      <c r="T60" s="20"/>
-      <c r="U60" s="20"/>
-      <c r="V60" s="20"/>
-      <c r="W60" s="20"/>
-      <c r="X60" s="20"/>
-      <c r="Y60" s="20"/>
-      <c r="Z60" s="20"/>
-      <c r="AA60" s="20"/>
-      <c r="AB60" s="20"/>
-      <c r="AC60" s="20"/>
-      <c r="AD60" s="20"/>
-      <c r="AE60" s="20"/>
-      <c r="AF60" s="20"/>
-      <c r="AG60" s="20"/>
-      <c r="AH60" s="20"/>
-      <c r="AI60" s="20"/>
-      <c r="AJ60" s="20"/>
-      <c r="AK60" s="20"/>
-    </row>
-    <row r="61" spans="1:41">
-      <c r="A61" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="B61" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-      <c r="K61" s="20"/>
-      <c r="L61" s="20"/>
-      <c r="M61" s="20"/>
-      <c r="N61" s="20"/>
-      <c r="O61" s="20"/>
-      <c r="P61" s="20"/>
-      <c r="Q61" s="20"/>
-      <c r="R61" s="20"/>
-      <c r="S61" s="20"/>
-      <c r="T61" s="20"/>
-      <c r="U61" s="20"/>
-      <c r="V61" s="20"/>
-      <c r="W61" s="20"/>
-      <c r="X61" s="20"/>
-      <c r="Y61" s="20"/>
-      <c r="Z61" s="20"/>
-      <c r="AA61" s="20"/>
-      <c r="AB61" s="20"/>
-      <c r="AC61" s="20"/>
-      <c r="AD61" s="20"/>
-      <c r="AE61" s="20"/>
-      <c r="AF61" s="20"/>
-      <c r="AG61" s="20"/>
-      <c r="AH61" s="20"/>
-      <c r="AI61" s="20"/>
-      <c r="AJ61" s="20"/>
-      <c r="AK61" s="20"/>
+      <c r="C61" s="19"/>
+      <c r="D61" s="19"/>
+      <c r="E61" s="19"/>
+      <c r="F61" s="19"/>
+      <c r="G61" s="19"/>
+      <c r="H61" s="19"/>
+      <c r="I61" s="19"/>
+      <c r="J61" s="19"/>
+      <c r="K61" s="19"/>
+      <c r="L61" s="19"/>
+      <c r="M61" s="19"/>
+      <c r="N61" s="19"/>
+      <c r="O61" s="19"/>
+      <c r="P61" s="19"/>
+      <c r="Q61" s="19"/>
+      <c r="R61" s="19"/>
+      <c r="S61" s="19"/>
+      <c r="T61" s="19"/>
+      <c r="U61" s="19"/>
+      <c r="V61" s="19"/>
+      <c r="W61" s="19"/>
+      <c r="X61" s="19"/>
+      <c r="Y61" s="19"/>
+      <c r="Z61" s="19"/>
+      <c r="AA61" s="19"/>
+      <c r="AB61" s="19"/>
+      <c r="AC61" s="19"/>
+      <c r="AD61" s="19"/>
+      <c r="AE61" s="19"/>
+      <c r="AF61" s="19"/>
+      <c r="AG61" s="19"/>
+      <c r="AH61" s="19"/>
+      <c r="AI61" s="19"/>
+      <c r="AJ61" s="19"/>
+      <c r="AK61" s="19"/>
     </row>
     <row r="62" spans="1:41">
-      <c r="A62" s="20"/>
-      <c r="B62" s="20"/>
-      <c r="C62" s="20"/>
-      <c r="D62" s="20"/>
-      <c r="E62" s="20"/>
-      <c r="F62" s="20"/>
-      <c r="G62" s="20"/>
-      <c r="H62" s="20"/>
-      <c r="I62" s="20"/>
-      <c r="J62" s="20"/>
-      <c r="K62" s="20"/>
-      <c r="L62" s="20"/>
-      <c r="M62" s="20"/>
-      <c r="N62" s="20"/>
-      <c r="O62" s="20"/>
-      <c r="P62" s="20"/>
-      <c r="Q62" s="20"/>
-      <c r="R62" s="20"/>
-      <c r="S62" s="20"/>
-      <c r="T62" s="20"/>
-      <c r="U62" s="20"/>
-      <c r="V62" s="20"/>
-      <c r="W62" s="20"/>
-      <c r="X62" s="20"/>
-      <c r="Y62" s="20"/>
-      <c r="Z62" s="20"/>
-      <c r="AA62" s="20"/>
-      <c r="AB62" s="20"/>
-      <c r="AC62" s="20"/>
-      <c r="AD62" s="20"/>
-      <c r="AE62" s="20"/>
-      <c r="AF62" s="20"/>
-      <c r="AG62" s="20"/>
-      <c r="AH62" s="20"/>
-      <c r="AI62" s="20"/>
-      <c r="AJ62" s="20"/>
-      <c r="AK62" s="20"/>
+      <c r="A62" s="19"/>
+      <c r="B62" s="19"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="19"/>
+      <c r="J62" s="19"/>
+      <c r="K62" s="19"/>
+      <c r="L62" s="19"/>
+      <c r="M62" s="19"/>
+      <c r="N62" s="19"/>
+      <c r="O62" s="19"/>
+      <c r="P62" s="19"/>
+      <c r="Q62" s="19"/>
+      <c r="R62" s="19"/>
+      <c r="S62" s="19"/>
+      <c r="T62" s="19"/>
+      <c r="U62" s="19"/>
+      <c r="V62" s="19"/>
+      <c r="W62" s="19"/>
+      <c r="X62" s="19"/>
+      <c r="Y62" s="19"/>
+      <c r="Z62" s="19"/>
+      <c r="AA62" s="19"/>
+      <c r="AB62" s="19"/>
+      <c r="AC62" s="19"/>
+      <c r="AD62" s="19"/>
+      <c r="AE62" s="19"/>
+      <c r="AF62" s="19"/>
+      <c r="AG62" s="19"/>
+      <c r="AH62" s="19"/>
+      <c r="AI62" s="19"/>
+      <c r="AJ62" s="19"/>
+      <c r="AK62" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A2:Z2"/>
+    <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="A2:AO2"/>
     <mergeCell ref="A47:G47"/>
     <mergeCell ref="A57:G57"/>
   </mergeCells>

</xml_diff>